<commit_message>
chore(lab): reset generated outputs for guided video practice
Archive build/logs/waves with integrity inventories, preserve 65 existing working logs as a labeled historical snapshot and ignore future runtime outputs. Add make clean and a guided study/video route in the current workspace. Retarget recorded ISA evidence links without changing results. Checked cleanup on fixtures, hashes, CSV/XLSX, links and Make previews; no RTL tests or physical flow run. Preserve user Makefile spacing outside this commit.
</commit_message>
<xml_diff>
--- a/docs/isa/coverage.xlsx
+++ b/docs/isa/coverage.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M5" s="0" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M8" s="0" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M9" s="0" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M10" s="0" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="L11" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M11" s="0" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M12" s="0" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M13" s="0" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M14" s="0" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M15" s="0" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M16" s="0" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M17" s="0" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M18" s="0" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L19" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M19" s="0" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_alu.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M20" s="0" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_pc.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_pc.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M21" s="0" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_pc.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_pc.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M22" s="0" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M23" s="0" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M24" s="0" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="L25" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M25" s="0" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M26" s="0" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L27" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M27" s="0" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="L28" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_branch_comp.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M28" s="0" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_pc.log; results/logs/tb_imm_ext.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_pc.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M29" s="0" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="L30" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_pc.log; results/logs/tb_imm_ext.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_pc.log; results/history/pre-guided-20261017/logs/tb_imm_ext.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M30" s="0" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="L31" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M31" s="0" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M32" s="0" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M33" s="0" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M34" s="0" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M35" s="0" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M36" s="0" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M37" s="0" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_lsu.log; results/history/pre-guided-20261017/logs/tb_dmem.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M38" s="0" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="L39" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_multiplier.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M39" s="0" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="L40" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_multiplier.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M40" s="0" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_multiplier.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M41" s="0" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="L42" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/history/pre-guided-20261017/logs/tb_decoder.log; results/history/pre-guided-20261017/logs/tb_multiplier.log; results/history/pre-guided-20261017/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M42" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix(crc): match official Xicrc contract and validate stage 2 firmware
Use rs1 for data and rs2 for the previous CRC16; process selected bytes
most significant first. Preserve encodings and the multicycle FSM, enable
Xicrc by default, and keep the historical parameter as an opt-out.

Add SHA-pinned official image preparation and a terminal-write/loop test,
including dynamic coverage of 44 instruction types. Update reference
models, own firmware, coverage, labs, module diagrams and the v0.6 report.
Archive reproducible regression logs, official VCD and a checked waveform.

Validation: 32 RTL testbenches and lint for both tops PASS; 18,304 CRC
vectors; 88,727 ISA retirements. Official firmware PASS: 252 retirements,
1,026 cycles, 16 CRC operations and three terminal-loop commits. Negative
test rejects the pre-fix CRC. Image integrity tests and report checks PASS.
No synthesis or physical implementation was run for this revision.
</commit_message>
<xml_diff>
--- a/docs/isa/coverage.xlsx
+++ b/docs/isa/coverage.xlsx
@@ -313,13 +313,13 @@
         </is>
       </c>
       <c r="B11" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C11" s="0">
         <v>3</v>
       </c>
       <c r="D11" s="4">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="12">
@@ -345,13 +345,13 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2">
         <v>47</v>
       </c>
       <c r="D13" s="6">
-        <v>0.8723404255319149</v>
+        <v>0.9361702127659575</v>
       </c>
     </row>
     <row r="14"/>
@@ -363,7 +363,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>41/47 instruções</t>
+          <t>44/47 instruções</t>
         </is>
       </c>
     </row>
@@ -373,9 +373,9 @@
           <t>Firmware oficial</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -531,24 +531,24 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
-          <t>64010 aposentadorias no teste próprio</t>
+          <t>74378 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -598,19 +598,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -665,19 +665,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -732,19 +732,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M5" s="0" t="inlineStr">
@@ -799,19 +799,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -866,19 +866,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
@@ -933,19 +933,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M8" s="0" t="inlineStr">
@@ -1000,19 +1000,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M9" s="0" t="inlineStr">
@@ -1067,19 +1067,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M10" s="0" t="inlineStr">
@@ -1134,19 +1134,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L11" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M11" s="0" t="inlineStr">
@@ -1201,24 +1201,24 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M12" s="0" t="inlineStr">
         <is>
-          <t>10779 aposentadorias no teste próprio</t>
+          <t>12507 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -1268,19 +1268,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M13" s="0" t="inlineStr">
@@ -1335,19 +1335,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M14" s="0" t="inlineStr">
@@ -1402,19 +1402,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M15" s="0" t="inlineStr">
@@ -1469,19 +1469,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M16" s="0" t="inlineStr">
@@ -1536,19 +1536,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M17" s="0" t="inlineStr">
@@ -1603,19 +1603,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M18" s="0" t="inlineStr">
@@ -1670,19 +1670,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K19" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L19" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M19" s="0" t="inlineStr">
@@ -1737,19 +1737,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_alu.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M20" s="0" t="inlineStr">
@@ -1804,19 +1804,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_pc.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M21" s="0" t="inlineStr">
@@ -1871,19 +1871,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_imm_ext.log; results/logs/tb_pc.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M22" s="0" t="inlineStr">
@@ -1938,19 +1938,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M23" s="0" t="inlineStr">
@@ -2005,19 +2005,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M24" s="0" t="inlineStr">
@@ -2072,19 +2072,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K25" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L25" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M25" s="0" t="inlineStr">
@@ -2139,19 +2139,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M26" s="0" t="inlineStr">
@@ -2206,19 +2206,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K27" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L27" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M27" s="0" t="inlineStr">
@@ -2273,19 +2273,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K28" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L28" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_branch_comp.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M28" s="0" t="inlineStr">
@@ -2340,19 +2340,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_pc.log; results/logs/tb_imm_ext.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M29" s="0" t="inlineStr">
@@ -2407,19 +2407,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K30" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L30" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_pc.log; results/logs/tb_imm_ext.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M30" s="0" t="inlineStr">
@@ -2474,19 +2474,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K31" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L31" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M31" s="0" t="inlineStr">
@@ -2541,19 +2541,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M32" s="0" t="inlineStr">
@@ -2608,19 +2608,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M33" s="0" t="inlineStr">
@@ -2675,19 +2675,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M34" s="0" t="inlineStr">
@@ -2742,19 +2742,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M35" s="0" t="inlineStr">
@@ -2809,19 +2809,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M36" s="0" t="inlineStr">
@@ -2876,19 +2876,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M37" s="0" t="inlineStr">
@@ -2943,19 +2943,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_lsu.log; results/logs/tb_dmem.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M38" s="0" t="inlineStr">
@@ -3010,19 +3010,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K39" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L39" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M39" s="0" t="inlineStr">
@@ -3077,19 +3077,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K40" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L40" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M40" s="0" t="inlineStr">
@@ -3144,19 +3144,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K41" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M41" s="0" t="inlineStr">
@@ -3211,19 +3211,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K42" s="0" t="inlineStr">
         <is>
-          <t>isa-41-v1</t>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L42" s="0" t="inlineStr">
         <is>
-          <t>results/logs/tb_decoder.log; results/logs/tb_multiplier.log; results/logs/tb_isa.log</t>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M42" s="0" t="inlineStr">
@@ -3258,44 +3258,44 @@
           <t>1000000</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I43" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J43" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>crc</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K43" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L43" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M43" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>74 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -3325,44 +3325,44 @@
           <t>1000000</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H44" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I44" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>crc</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K44" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L44" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M44" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>74 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -3392,44 +3392,44 @@
           <t>1000000</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I45" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>crc</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K45" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-44-v1</t>
         </is>
       </c>
       <c r="L45" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M45" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>74 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(system): complete 47-instruction profile with precise EEI traps
Implement ordered FENCE and exact ECALL/EBREAK decoding with a terminal TRAP state, separate from illegal-instruction FAULT. Expose trap type and PC through core/top and preserve the reduced simple_system interface.

Validate 33 RTL testbenches and both lint tops, 512 FENCE executions, 256 traps per instruction, reset recovery, and the unchanged official firmware (44 types). Reject stale or inflated coverage, archive manifests/logs/VCD, and update the 12-page report and labs. No synthesis or physical signoff performed.
</commit_message>
<xml_diff>
--- a/docs/isa/coverage.xlsx
+++ b/docs/isa/coverage.xlsx
@@ -329,13 +329,13 @@
         </is>
       </c>
       <c r="B12" s="0">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C12" s="0">
         <v>3</v>
       </c>
       <c r="D12" s="4">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -345,13 +345,13 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2">
         <v>47</v>
       </c>
       <c r="D13" s="6">
-        <v>0.9361702127659575</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="14"/>
@@ -363,7 +363,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>44/47 instruções</t>
+          <t>47/47 instruções</t>
         </is>
       </c>
     </row>
@@ -375,7 +375,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>44/47 tipos com PASS; demais conforme tabela</t>
         </is>
       </c>
     </row>
@@ -387,7 +387,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>O firmware próprio não substitui a validação oficial.</t>
+          <t>Sistema: testes próprios e contrato EEI CMOS; traps não aposentam.</t>
         </is>
       </c>
     </row>
@@ -538,17 +538,17 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
-          <t>74378 aposentadorias no teste próprio</t>
+          <t>74426 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -605,12 +605,12 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M5" s="0" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
@@ -940,12 +940,12 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M8" s="0" t="inlineStr">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M9" s="0" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L10" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M10" s="0" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L11" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M11" s="0" t="inlineStr">
@@ -1208,17 +1208,17 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M12" s="0" t="inlineStr">
         <is>
-          <t>12507 aposentadorias no teste próprio</t>
+          <t>12515 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -1275,12 +1275,12 @@
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M13" s="0" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M14" s="0" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M15" s="0" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M16" s="0" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M17" s="0" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M18" s="0" t="inlineStr">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="K19" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L19" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M19" s="0" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_alu.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_alu.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M20" s="0" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_pc.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M21" s="0" t="inlineStr">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_pc.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M22" s="0" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M23" s="0" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M24" s="0" t="inlineStr">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="K25" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L25" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M25" s="0" t="inlineStr">
@@ -2146,12 +2146,12 @@
       </c>
       <c r="K26" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L26" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M26" s="0" t="inlineStr">
@@ -2213,12 +2213,12 @@
       </c>
       <c r="K27" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L27" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M27" s="0" t="inlineStr">
@@ -2280,12 +2280,12 @@
       </c>
       <c r="K28" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L28" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_branch_comp.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_branch_comp.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M28" s="0" t="inlineStr">
@@ -2347,12 +2347,12 @@
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_pc.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M29" s="0" t="inlineStr">
@@ -2414,12 +2414,12 @@
       </c>
       <c r="K30" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L30" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_pc.log; results/experiments/crc-official-20261027/logs/tb_imm_ext.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_pc.log; results/experiments/isa-47-20261027/logs/tb_imm_ext.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M30" s="0" t="inlineStr">
@@ -2481,12 +2481,12 @@
       </c>
       <c r="K31" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L31" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M31" s="0" t="inlineStr">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M32" s="0" t="inlineStr">
@@ -2615,17 +2615,17 @@
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M33" s="0" t="inlineStr">
         <is>
-          <t>23 aposentadorias no teste próprio</t>
+          <t>28 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2682,12 @@
       </c>
       <c r="K34" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L34" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M34" s="0" t="inlineStr">
@@ -2749,12 +2749,12 @@
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M35" s="0" t="inlineStr">
@@ -2816,12 +2816,12 @@
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M36" s="0" t="inlineStr">
@@ -2883,12 +2883,12 @@
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M37" s="0" t="inlineStr">
@@ -2950,17 +2950,17 @@
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_lsu.log; results/experiments/crc-official-20261027/logs/tb_dmem.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_lsu.log; results/experiments/isa-47-20261027/logs/tb_dmem.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M38" s="0" t="inlineStr">
         <is>
-          <t>35 aposentadorias no teste próprio</t>
+          <t>36 aposentadorias no teste próprio</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3017,12 @@
       </c>
       <c r="K39" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L39" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_multiplier.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M39" s="0" t="inlineStr">
@@ -3084,12 +3084,12 @@
       </c>
       <c r="K40" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L40" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_multiplier.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M40" s="0" t="inlineStr">
@@ -3151,12 +3151,12 @@
       </c>
       <c r="K41" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_multiplier.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M41" s="0" t="inlineStr">
@@ -3218,12 +3218,12 @@
       </c>
       <c r="K42" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L42" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_multiplier.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_multiplier.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M42" s="0" t="inlineStr">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="K43" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L43" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_crc.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M43" s="0" t="inlineStr">
@@ -3352,12 +3352,12 @@
       </c>
       <c r="K44" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L44" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_crc.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M44" s="0" t="inlineStr">
@@ -3419,12 +3419,12 @@
       </c>
       <c r="K45" s="0" t="inlineStr">
         <is>
-          <t>isa-44-v1</t>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L45" s="0" t="inlineStr">
         <is>
-          <t>results/experiments/crc-official-20261027/logs/tb_decoder.log; results/experiments/crc-official-20261027/logs/tb_crc.log; results/experiments/crc-official-20261027/logs/tb_isa.log; results/experiments/crc-official-20261027/logs/tb_official_firmware.log</t>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_crc.log; results/experiments/isa-47-20261027/logs/tb_isa.log; results/experiments/isa-47-20261027/logs/tb_official_firmware.log</t>
         </is>
       </c>
       <c r="M45" s="0" t="inlineStr">
@@ -3441,62 +3441,62 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>PENDENTE_1</t>
+          <t>FENCE</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
         <is>
+          <t>0001111</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="D46" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E46" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H46" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J46" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F46" s="0" t="inlineStr">
+        <is>
+          <t>decoder/control_unit/riscv_core</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J46" s="0" t="inlineStr">
+        <is>
+          <t>NÃO EXERCITADA</t>
         </is>
       </c>
       <c r="K46" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L46" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_control_unit.log; results/experiments/isa-47-20261027/logs/tb_core_system.log; results/experiments/isa-47-20261027/logs/tb_isa.log</t>
         </is>
       </c>
       <c r="M46" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>5 aposentadorias no teste próprio; contrato EEI CMOS, firmware publicado não exercita</t>
         </is>
       </c>
     </row>
@@ -3508,62 +3508,62 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>PENDENTE_2</t>
+          <t>ECALL</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
         <is>
+          <t>1110011</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="D47" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E47" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I47" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J47" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F47" s="0" t="inlineStr">
+        <is>
+          <t>decoder/control_unit/riscv_core</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J47" s="0" t="inlineStr">
+        <is>
+          <t>NÃO EXERCITADA</t>
         </is>
       </c>
       <c r="K47" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L47" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_control_unit.log; results/experiments/isa-47-20261027/logs/tb_core_system.log</t>
         </is>
       </c>
       <c r="M47" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>256 traps precisos verificados; não aposenta; contrato EEI CMOS, firmware publicado não exercita</t>
         </is>
       </c>
     </row>
@@ -3575,62 +3575,62 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>PENDENTE_3</t>
+          <t>EBREAK</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
         <is>
+          <t>1110011</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
           <t/>
         </is>
       </c>
-      <c r="D48" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E48" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="H48" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="I48" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>decoder/control_unit/riscv_core</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J48" s="0" t="inlineStr">
+        <is>
+          <t>NÃO EXERCITADA</t>
         </is>
       </c>
       <c r="K48" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>isa-47-v1</t>
         </is>
       </c>
       <c r="L48" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>results/experiments/isa-47-20261027/logs/tb_decoder.log; results/experiments/isa-47-20261027/logs/tb_control_unit.log; results/experiments/isa-47-20261027/logs/tb_core_system.log</t>
         </is>
       </c>
       <c r="M48" s="0" t="inlineStr">
         <is>
-          <t>Definição oficial pendente</t>
+          <t>256 traps precisos verificados; não aposenta; contrato EEI CMOS, firmware publicado não exercita</t>
         </is>
       </c>
     </row>

</xml_diff>